<commit_message>
DUI file: add expanded audit (CDX + Common Crawl sweeps across 120 .gov domains)
</commit_message>
<xml_diff>
--- a/dui_dwi_bodycam_cases.xlsx
+++ b/dui_dwi_bodycam_cases.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="135" customWidth="1" min="1" max="1"/>
@@ -545,52 +545,56 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>• Search engines (Bing/DDG): returned unrelated junk / rate-limited from this host; several rounds tried.</t>
+          <t>• Wayback CDX wildcard sweep across 120 city/county/sheriff .gov domains (dui/dwi/bodycam URL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>• All other agencies' DUI bodycam material (state patrols, LAPD, police departments) lives on</t>
+          <t xml:space="preserve">  patterns): 190 raw matches, 8 strict — all audit reports or internal redirect payloads, no case videos.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  YouTube or social media — excluded by rule.</t>
+          <t>• Common Crawl index sweep across the same 120 domains (matchType=domain): 0 DUI/DWI URLs</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (current indices no longer support server-side URL filtering; enumeration confirmed empty).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>CONCLUSION: Official non-YouTube DUI/DWI bodycam releases effectively do not exist as a category.</t>
+          <t>• Search engines (Bing/DDG/Brave/Ecosia/Mojeek/lite-DDG): returned unrelated junk / rate-limited</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DUI arrest footage is published almost exclusively on department YouTube channels and social media.</t>
+          <t xml:space="preserve">  from this host; several rounds tried.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>To build a real 100-case DUI file, the no-YouTube rule must be relaxed to allow official department</t>
+          <t>• All other agencies' DUI bodycam material (state patrols, LAPD, police departments) lives on</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>channels (host-verified, e.g. Sacramento Sheriff's own channel embedded on sacsheriff.com).</t>
+          <t xml:space="preserve">  YouTube or social media — excluded by rule.</t>
         </is>
       </c>
     </row>
@@ -600,19 +604,50 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Sheet 'Closest Verified Traffic Cases' lists the nearest matches that DO pass every other rule:</t>
+          <t>CONCLUSION: Official non-YouTube DUI/DWI bodycam releases effectively do not exist as a category.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>official traffic/motor-vehicle incident releases with BWC, combined over 15 minutes — clearly marked</t>
+          <t>DUI arrest footage is published almost exclusively on department YouTube channels and social media.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>To build a real 100-case DUI file, the no-YouTube rule must be relaxed to allow official department</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>channels (host-verified, e.g. Sacramento Sheriff's own channel embedded on sacsheriff.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Sheet 'Closest Verified Traffic Cases' lists the nearest matches that DO pass every other rule:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>official traffic/motor-vehicle incident releases with BWC, combined over 15 minutes — clearly marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>as NOT DUI-confirmed.</t>
         </is>

</xml_diff>